<commit_message>
Ausschluss von Inspektions-Tauschen (Ursache-Spalte) + Verschluss-Befund
- labels: Stoerungen header-basiert einlesen (robust); Spalten verlauf/ursache
- make_label_template: Spalte 'Ursache' (Verschleiss/Inspektion) mit Dropdown
- loso_model: schliesst faults mit ursache=Inspektion aus (sofern annotiert)

Diagnose: 3 von 5 Verschluss-Faellen zeigen KEIN Signal vor dem Datum
(roll_z_tt ~0.5) -> Kandidaten fuer turnusmaessige Tausche; vom Nutzer gegen
Akten zu pruefen, nicht automatisch ausschliessen (zirkulaer).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/labels/stoerungen_template.xlsx
+++ b/data/labels/stoerungen_template.xlsx
@@ -548,7 +548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -557,11 +557,13 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -597,25 +599,35 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>Verlauf</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Ursache</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
           <t>Komponente</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Schweregrad</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Sicherheit</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Quelle</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Notizen</t>
         </is>
@@ -654,42 +666,58 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
+          <t>graduell (langsam) oder abrupt (plötzlich) — abrupte sind nicht vorwarnbar</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Verschleiß oder Inspektion (Routine-Tausch) — Inspektion wird ausgeschlossen</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
           <t>z.B. Antrieb SAT01, falls bekannt</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Warnung / Störung / Ausfall</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>bestätigt oder vermutet</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Woher die Info stammt (DIANA, Instandhaltung, ...)</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>Freitext</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation sqref="E3:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"L,R,beide,unbekannt"</formula1>
     </dataValidation>
     <dataValidation sqref="F3:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Erhöhter Strom/Leistung Umlauf,Stark erhöhter Strom/Leistung Umlauf,Erhöhter Strom/Leistung Verriegelung,Stark erhöhter Strom/Leistung Verriegelung,Erhöhter Strom/Leistung Entriegelung,Stark erhöhter Strom/Leistung Entriegelung,Störung Endlage,Stark verlängerte Umlaufzeit,Abweichende Referenz,Sonstige/Unbekannt"</formula1>
     </dataValidation>
+    <dataValidation sqref="G3:G500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"graduell,abrupt,unbekannt"</formula1>
+    </dataValidation>
     <dataValidation sqref="H3:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Verschleiß,Inspektion,unbekannt"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J3:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Warnung,Störung,Ausfall,unbekannt"</formula1>
     </dataValidation>
-    <dataValidation sqref="I3:I500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K3:K500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"bestätigt,vermutet"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>